<commit_message>
Asesorias 11 y 16 de septiembre
</commit_message>
<xml_diff>
--- a/excels/Presupuesto SIRCOVA.xlsx
+++ b/excels/Presupuesto SIRCOVA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kennethram\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kennethram\Documents\GitHub\PropuestaProyectoDeCarrera\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4B0147-312B-4A19-96C8-DA128B2B8C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7676E1F8-9DF9-4852-A835-8EFE6683D34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -552,6 +552,45 @@
     <xf numFmtId="9" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="11" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -579,23 +618,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -610,33 +637,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="11" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -855,32 +855,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="56" customWidth="1"/>
+    <col min="1" max="1" width="33.8984375" customWidth="1"/>
+    <col min="2" max="2" width="13.69921875" customWidth="1"/>
+    <col min="3" max="3" width="12.69921875" customWidth="1"/>
+    <col min="4" max="4" width="46.296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
     </row>
     <row r="2" spans="1:4" ht="22.35" customHeight="1">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-    </row>
-    <row r="4" spans="1:4" ht="22.35" customHeight="1">
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+    </row>
+    <row r="4" spans="1:4" ht="27" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -895,12 +895,12 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="17.55" customHeight="1">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="50" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="38"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="40"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="52"/>
     </row>
     <row r="6" spans="1:4" ht="24" customHeight="1">
       <c r="A6" s="4" t="s">
@@ -1000,7 +1000,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="22.35" customHeight="1">
+    <row r="13" spans="1:4" ht="31.8" customHeight="1">
       <c r="A13" s="10" t="s">
         <v>25</v>
       </c>
@@ -1014,12 +1014,12 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="22.35" customHeight="1">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="41"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="40"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="52"/>
     </row>
     <row r="15" spans="1:4" ht="24" customHeight="1">
       <c r="A15" s="4" t="s">
@@ -1036,10 +1036,10 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="33.6" customHeight="1">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="45" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="20">
@@ -1050,27 +1050,27 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="24" customHeight="1">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C17" s="19">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="33.6" customHeight="1">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="36"/>
+      <c r="B18" s="49"/>
       <c r="C18" s="22">
         <f>SUM(C15:C17)</f>
-        <v>550</v>
+        <v>1450</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>35</v>
@@ -1080,8 +1080,8 @@
       <c r="A19" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="41"/>
-      <c r="C19" s="42"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="40"/>
       <c r="D19" s="38"/>
     </row>
     <row r="20" spans="1:4" ht="33.6" customHeight="1">
@@ -1118,7 +1118,7 @@
       <c r="B22" s="11"/>
       <c r="C22" s="21">
         <f>SUM(C13,C18,C21)</f>
-        <v>57870</v>
+        <v>58770</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>43</v>
@@ -1131,7 +1131,7 @@
       <c r="B23" s="16"/>
       <c r="C23" s="23">
         <f>15%*(C13+C18)</f>
-        <v>280.5</v>
+        <v>415.5</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>45</v>
@@ -1144,7 +1144,7 @@
       <c r="B24" s="18"/>
       <c r="C24" s="24">
         <f>C22+C23</f>
-        <v>58150.5</v>
+        <v>59185.5</v>
       </c>
       <c r="D24" s="17" t="s">
         <v>47</v>
@@ -1152,12 +1152,17 @@
     </row>
     <row r="25" spans="1:4" ht="7.95" customHeight="1"/>
     <row r="26" spans="1:4" ht="17.55" customHeight="1">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="D28">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1188,20 +1193,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
     </row>
     <row r="2" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A2" s="45"/>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
+      <c r="A2" s="54"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
     </row>
     <row r="3" spans="1:5" ht="27.6">
       <c r="A3" s="25" t="s">
@@ -1221,57 +1226,57 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="54.6" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="54" t="s">
+      <c r="C4" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="30">
         <f>Presupuesto!C24-Presupuesto!C21</f>
-        <v>2150.5</v>
-      </c>
-      <c r="E4" s="56">
+        <v>3185.5</v>
+      </c>
+      <c r="E4" s="36">
         <f>D4/$D$7</f>
-        <v>3.6981625265474931E-2</v>
+        <v>5.382230444956957E-2</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="65.400000000000006" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="49" t="s">
+      <c r="B5" s="29" t="s">
         <v>58</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="49">
+      <c r="D5" s="29">
         <f>Presupuesto!C21</f>
         <v>56000</v>
       </c>
-      <c r="E5" s="57">
+      <c r="E5" s="37">
         <f>D5/$D$7</f>
-        <v>0.96301837473452512</v>
+        <v>0.94617769555043041</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="72" customHeight="1">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="53" t="s">
+      <c r="C6" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="52">
+      <c r="D6" s="32">
         <v>0</v>
       </c>
-      <c r="E6" s="52">
+      <c r="E6" s="32">
         <f>0</f>
         <v>0</v>
       </c>
@@ -1284,7 +1289,7 @@
       <c r="C7" s="26"/>
       <c r="D7" s="27">
         <f>Presupuesto!C24</f>
-        <v>58150.5</v>
+        <v>59185.5</v>
       </c>
       <c r="E7" s="28">
         <f>1</f>
@@ -1292,42 +1297,42 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="41.4" customHeight="1">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="48"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1"/>
     <row r="10" spans="1:5" ht="24" customHeight="1">
-      <c r="A10" s="46"/>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
+      <c r="A10" s="55"/>
+      <c r="B10" s="55"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="55"/>
+      <c r="E10" s="55"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="46"/>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
+      <c r="A11" s="55"/>
+      <c r="B11" s="55"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="55"/>
     </row>
     <row r="12" spans="1:5" ht="24" customHeight="1">
-      <c r="A12" s="46"/>
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="46"/>
+      <c r="A12" s="55"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
     </row>
     <row r="13" spans="1:5" ht="24" customHeight="1">
-      <c r="A13" s="46"/>
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="46"/>
+      <c r="A13" s="55"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
     </row>
     <row r="14" spans="1:5" ht="24" customHeight="1"/>
     <row r="15" spans="1:5" ht="24" customHeight="1"/>

</xml_diff>